<commit_message>
Updating for developing online viewing
</commit_message>
<xml_diff>
--- a/output/ntl_summary_tables.xlsx
+++ b/output/ntl_summary_tables.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Region_Pixels" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="City_Radiance" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="City_Pixels" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Logged_Somaliland_Radiance" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2143,4 +2144,126 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>logged_radiance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2012</v>
+      </c>
+      <c r="B2" t="n">
+        <v>7.452750418518224</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2013</v>
+      </c>
+      <c r="B3" t="n">
+        <v>7.488461380196333</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2014</v>
+      </c>
+      <c r="B4" t="n">
+        <v>7.578707974032314</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2015</v>
+      </c>
+      <c r="B5" t="n">
+        <v>7.680360380876798</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2016</v>
+      </c>
+      <c r="B6" t="n">
+        <v>7.753022507602916</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2017</v>
+      </c>
+      <c r="B7" t="n">
+        <v>7.915968641206629</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B8" t="n">
+        <v>8.165164579397244</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B9" t="n">
+        <v>8.371612352049818</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B10" t="n">
+        <v>8.637905266578501</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B11" t="n">
+        <v>8.961943113187305</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B12" t="n">
+        <v>9.183154152931865</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B13" t="n">
+        <v>9.286263837980318</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>